<commit_message>
STM32 product selector bug fixes and format change
</commit_message>
<xml_diff>
--- a/product_selector_out/STM32 wireless MCUs - diff.xlsx
+++ b/product_selector_out/STM32 wireless MCUs - diff.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Diff" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Diff'!$A$18:$E$211</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Diff'!$A$18:$E$212</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E211"/>
+  <dimension ref="A1:E212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -617,7 +617,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>6239</v>
+        <v>6238</v>
       </c>
     </row>
     <row r="18">
@@ -5052,18 +5052,22 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Longevity Commitment (yr) typ</t>
-        </is>
-      </c>
-      <c r="C210" t="inlineStr"/>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E210" s="3" t="inlineStr">
-        <is>
-          <t>ADDED_COLUMN</t>
+          <t>Arm Cortex-M0+</t>
+        </is>
+      </c>
+      <c r="E210" s="4" t="inlineStr">
+        <is>
+          <t>BLANK_FILLED</t>
         </is>
       </c>
     </row>
@@ -5075,13 +5079,13 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Longevity Starting Date</t>
+          <t>Longevity Commitment (yr) typ</t>
         </is>
       </c>
       <c r="C211" t="inlineStr"/>
       <c r="D211" t="inlineStr">
         <is>
-          <t>2026-01-01T00:00:00.000+01:00</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E211" s="3" t="inlineStr">
@@ -5090,8 +5094,31 @@
         </is>
       </c>
     </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>STM32WB05TN</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Longevity Starting Date</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr"/>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>2026-01-01T00:00:00.000+01:00</t>
+        </is>
+      </c>
+      <c r="E212" s="3" t="inlineStr">
+        <is>
+          <t>ADDED_COLUMN</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A18:E211"/>
+  <autoFilter ref="A18:E212"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
STM32 product selector bug fixes
</commit_message>
<xml_diff>
--- a/product_selector_out/STM32 wireless MCUs - diff.xlsx
+++ b/product_selector_out/STM32 wireless MCUs - diff.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Diff" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Diff'!$A$18:$E$212</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Diff'!$A$18:$E$218</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -33,7 +33,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -48,6 +48,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B7E1CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
     <fill>
@@ -71,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -79,6 +94,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -444,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E212"/>
+  <dimension ref="A1:E218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -537,7 +555,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -597,7 +615,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -607,7 +625,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -617,7 +635,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>6238</v>
+        <v>6236</v>
       </c>
     </row>
     <row r="18">
@@ -4197,18 +4215,22 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Longevity Commitment (yr) typ</t>
-        </is>
-      </c>
-      <c r="C173" t="inlineStr"/>
+          <t>Timers (16-bit) typ</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>3||5</t>
+        </is>
+      </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E173" s="3" t="inlineStr">
-        <is>
-          <t>ADDED_COLUMN</t>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E173" s="4" t="inlineStr">
+        <is>
+          <t>CHANGED</t>
         </is>
       </c>
     </row>
@@ -4220,59 +4242,67 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Longevity Starting Date</t>
-        </is>
-      </c>
-      <c r="C174" t="inlineStr"/>
+          <t>Timers (16-bit) typ</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>3, 5</t>
+        </is>
+      </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>2026-01-01T00:00:00.000+01:00</t>
-        </is>
-      </c>
-      <c r="E174" s="3" t="inlineStr">
-        <is>
-          <t>ADDED_COLUMN</t>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E174" s="5" t="inlineStr">
+        <is>
+          <t>DATASHEET_OVERRIDES_API</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>STM32WB55CC</t>
+          <t>STM32WB55VE</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Longevity Commitment (yr) typ</t>
-        </is>
-      </c>
-      <c r="C175" t="inlineStr"/>
+          <t>Timers (16-bit) typ</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>3||5 (workbook and API agree)</t>
+        </is>
+      </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E175" s="3" t="inlineStr">
-        <is>
-          <t>ADDED_COLUMN</t>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E175" s="6" t="inlineStr">
+        <is>
+          <t>ORIGINAL_MATCHED_API_NOT_DATASHEET</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>STM32WB55CC</t>
+          <t>STM32WB55VE</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Longevity Starting Date</t>
+          <t>Longevity Commitment (yr) typ</t>
         </is>
       </c>
       <c r="C176" t="inlineStr"/>
       <c r="D176" t="inlineStr">
         <is>
-          <t>2026-01-01T00:00:00.000+01:00</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E176" s="3" t="inlineStr">
@@ -4284,18 +4314,18 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>STM32WB55RE</t>
+          <t>STM32WB55VE</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Longevity Commitment (yr) typ</t>
+          <t>Longevity Starting Date</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
       <c r="D177" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2026-01-01T00:00:00.000+01:00</t>
         </is>
       </c>
       <c r="E177" s="3" t="inlineStr">
@@ -4307,18 +4337,18 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>STM32WB55RE</t>
+          <t>STM32WB55CC</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Longevity Starting Date</t>
+          <t>Longevity Commitment (yr) typ</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
       <c r="D178" t="inlineStr">
         <is>
-          <t>2026-01-01T00:00:00.000+01:00</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E178" s="3" t="inlineStr">
@@ -4330,18 +4360,18 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>STM32WB55VC</t>
+          <t>STM32WB55CC</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Longevity Commitment (yr) typ</t>
+          <t>Longevity Starting Date</t>
         </is>
       </c>
       <c r="C179" t="inlineStr"/>
       <c r="D179" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2026-01-01T00:00:00.000+01:00</t>
         </is>
       </c>
       <c r="E179" s="3" t="inlineStr">
@@ -4353,18 +4383,18 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>STM32WB55VC</t>
+          <t>STM32WB55RE</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Longevity Starting Date</t>
+          <t>Longevity Commitment (yr) typ</t>
         </is>
       </c>
       <c r="C180" t="inlineStr"/>
       <c r="D180" t="inlineStr">
         <is>
-          <t>2026-01-01T00:00:00.000+01:00</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E180" s="3" t="inlineStr">
@@ -4376,18 +4406,18 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>STM32WB55CG</t>
+          <t>STM32WB55RE</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Longevity Commitment (yr) typ</t>
+          <t>Longevity Starting Date</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
       <c r="D181" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2026-01-01T00:00:00.000+01:00</t>
         </is>
       </c>
       <c r="E181" s="3" t="inlineStr">
@@ -4399,76 +4429,88 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>STM32WB55CG</t>
+          <t>STM32WB55VC</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Longevity Starting Date</t>
-        </is>
-      </c>
-      <c r="C182" t="inlineStr"/>
+          <t>Timers (16-bit) typ</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>3||5</t>
+        </is>
+      </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>2026-01-01T00:00:00.000+01:00</t>
-        </is>
-      </c>
-      <c r="E182" s="3" t="inlineStr">
-        <is>
-          <t>ADDED_COLUMN</t>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E182" s="4" t="inlineStr">
+        <is>
+          <t>CHANGED</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>STM32WB55RG</t>
+          <t>STM32WB55VC</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Longevity Commitment (yr) typ</t>
-        </is>
-      </c>
-      <c r="C183" t="inlineStr"/>
+          <t>Timers (16-bit) typ</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>3, 5</t>
+        </is>
+      </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E183" s="3" t="inlineStr">
-        <is>
-          <t>ADDED_COLUMN</t>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E183" s="5" t="inlineStr">
+        <is>
+          <t>DATASHEET_OVERRIDES_API</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>STM32WB55RG</t>
+          <t>STM32WB55VC</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Longevity Starting Date</t>
-        </is>
-      </c>
-      <c r="C184" t="inlineStr"/>
+          <t>Timers (16-bit) typ</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>3||5 (workbook and API agree)</t>
+        </is>
+      </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>2026-01-01T00:00:00.000+01:00</t>
-        </is>
-      </c>
-      <c r="E184" s="3" t="inlineStr">
-        <is>
-          <t>ADDED_COLUMN</t>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E184" s="6" t="inlineStr">
+        <is>
+          <t>ORIGINAL_MATCHED_API_NOT_DATASHEET</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>STM32WB35CE</t>
+          <t>STM32WB55VC</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4491,7 +4533,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>STM32WB35CE</t>
+          <t>STM32WB55VC</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4514,7 +4556,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>STM32WB35CC</t>
+          <t>STM32WB55CG</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -4537,7 +4579,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>STM32WB35CC</t>
+          <t>STM32WB55CG</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -4560,7 +4602,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>STM32WB55CE</t>
+          <t>STM32WB55RG</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -4583,7 +4625,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>STM32WB55CE</t>
+          <t>STM32WB55RG</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -4606,7 +4648,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>STM32WB06CC</t>
+          <t>STM32WB35CE</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -4629,7 +4671,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>STM32WB06CC</t>
+          <t>STM32WB35CE</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -4652,7 +4694,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>STM32WB09KE</t>
+          <t>STM32WB35CC</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -4675,7 +4717,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>STM32WB09KE</t>
+          <t>STM32WB35CC</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -4698,7 +4740,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>STM32WB05KZ</t>
+          <t>STM32WB55CE</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -4721,7 +4763,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>STM32WB05KZ</t>
+          <t>STM32WB55CE</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -4744,7 +4786,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>STM32WB06KC</t>
+          <t>STM32WB06CC</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -4767,7 +4809,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>STM32WB06KC</t>
+          <t>STM32WB06CC</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -4790,7 +4832,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>STM32WB07CC</t>
+          <t>STM32WB09KE</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -4813,7 +4855,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>STM32WB07CC</t>
+          <t>STM32WB09KE</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -4836,7 +4878,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>STM32WB05TZ</t>
+          <t>STM32WB05KZ</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -4859,7 +4901,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>STM32WB05TZ</t>
+          <t>STM32WB05KZ</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -4882,7 +4924,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>STM32WB07KC</t>
+          <t>STM32WB06KC</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -4905,7 +4947,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>STM32WB07KC</t>
+          <t>STM32WB06KC</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -4928,45 +4970,41 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>STM32WB05KN</t>
+          <t>STM32WB07CC</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="C205" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>Longevity Commitment (yr) typ</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr"/>
       <c r="D205" t="inlineStr">
         <is>
-          <t>Arm Cortex-M0+</t>
-        </is>
-      </c>
-      <c r="E205" s="4" t="inlineStr">
-        <is>
-          <t>BLANK_FILLED</t>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E205" s="3" t="inlineStr">
+        <is>
+          <t>ADDED_COLUMN</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>STM32WB05KN</t>
+          <t>STM32WB07CC</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Longevity Commitment (yr) typ</t>
+          <t>Longevity Starting Date</t>
         </is>
       </c>
       <c r="C206" t="inlineStr"/>
       <c r="D206" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2026-01-01T00:00:00.000+01:00</t>
         </is>
       </c>
       <c r="E206" s="3" t="inlineStr">
@@ -4978,18 +5016,18 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>STM32WB05KN</t>
+          <t>STM32WB05TZ</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Longevity Starting Date</t>
+          <t>Longevity Commitment (yr) typ</t>
         </is>
       </c>
       <c r="C207" t="inlineStr"/>
       <c r="D207" t="inlineStr">
         <is>
-          <t>2026-01-01T00:00:00.000+01:00</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E207" s="3" t="inlineStr">
@@ -5001,18 +5039,18 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>STM32WB09TE</t>
+          <t>STM32WB05TZ</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Longevity Commitment (yr) typ</t>
+          <t>Longevity Starting Date</t>
         </is>
       </c>
       <c r="C208" t="inlineStr"/>
       <c r="D208" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2026-01-01T00:00:00.000+01:00</t>
         </is>
       </c>
       <c r="E208" s="3" t="inlineStr">
@@ -5024,18 +5062,18 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>STM32WB09TE</t>
+          <t>STM32WB07KC</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Longevity Starting Date</t>
+          <t>Longevity Commitment (yr) typ</t>
         </is>
       </c>
       <c r="C209" t="inlineStr"/>
       <c r="D209" t="inlineStr">
         <is>
-          <t>2026-01-01T00:00:00.000+01:00</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E209" s="3" t="inlineStr">
@@ -5047,68 +5085,68 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>STM32WB05TN</t>
+          <t>STM32WB07KC</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="C210" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>Longevity Starting Date</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr"/>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Arm Cortex-M0+</t>
-        </is>
-      </c>
-      <c r="E210" s="4" t="inlineStr">
-        <is>
-          <t>BLANK_FILLED</t>
+          <t>2026-01-01T00:00:00.000+01:00</t>
+        </is>
+      </c>
+      <c r="E210" s="3" t="inlineStr">
+        <is>
+          <t>ADDED_COLUMN</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>STM32WB05TN</t>
+          <t>STM32WB05KN</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Longevity Commitment (yr) typ</t>
-        </is>
-      </c>
-      <c r="C211" t="inlineStr"/>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E211" s="3" t="inlineStr">
-        <is>
-          <t>ADDED_COLUMN</t>
+          <t>Arm Cortex-M0+</t>
+        </is>
+      </c>
+      <c r="E211" s="7" t="inlineStr">
+        <is>
+          <t>BLANK_FILLED</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>STM32WB05TN</t>
+          <t>STM32WB05KN</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Longevity Starting Date</t>
+          <t>Longevity Commitment (yr) typ</t>
         </is>
       </c>
       <c r="C212" t="inlineStr"/>
       <c r="D212" t="inlineStr">
         <is>
-          <t>2026-01-01T00:00:00.000+01:00</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E212" s="3" t="inlineStr">
@@ -5117,8 +5155,150 @@
         </is>
       </c>
     </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>STM32WB05KN</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Longevity Starting Date</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr"/>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>2026-01-01T00:00:00.000+01:00</t>
+        </is>
+      </c>
+      <c r="E213" s="3" t="inlineStr">
+        <is>
+          <t>ADDED_COLUMN</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>STM32WB09TE</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Longevity Commitment (yr) typ</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr"/>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E214" s="3" t="inlineStr">
+        <is>
+          <t>ADDED_COLUMN</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>STM32WB09TE</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Longevity Starting Date</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr"/>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>2026-01-01T00:00:00.000+01:00</t>
+        </is>
+      </c>
+      <c r="E215" s="3" t="inlineStr">
+        <is>
+          <t>ADDED_COLUMN</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>STM32WB05TN</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Arm Cortex-M0+</t>
+        </is>
+      </c>
+      <c r="E216" s="7" t="inlineStr">
+        <is>
+          <t>BLANK_FILLED</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>STM32WB05TN</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Longevity Commitment (yr) typ</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr"/>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E217" s="3" t="inlineStr">
+        <is>
+          <t>ADDED_COLUMN</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>STM32WB05TN</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Longevity Starting Date</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr"/>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>2026-01-01T00:00:00.000+01:00</t>
+        </is>
+      </c>
+      <c r="E218" s="3" t="inlineStr">
+        <is>
+          <t>ADDED_COLUMN</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A18:E212"/>
+  <autoFilter ref="A18:E218"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
STM32 product selector LPUART
</commit_message>
<xml_diff>
--- a/product_selector_out/STM32 wireless MCUs - diff.xlsx
+++ b/product_selector_out/STM32 wireless MCUs - diff.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Diff" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Diff'!$A$18:$E$218</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Diff'!$A$18:$E$211</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -33,7 +33,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -48,21 +48,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00B7E1CD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
     <fill>
@@ -86,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -94,9 +79,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -462,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E218"/>
+  <dimension ref="A1:E211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -555,7 +537,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -565,7 +547,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -615,7 +597,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -625,7 +607,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -635,7 +617,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>6236</v>
+        <v>6239</v>
       </c>
     </row>
     <row r="18">
@@ -4215,22 +4197,18 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Timers (16-bit) typ</t>
-        </is>
-      </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>3||5</t>
-        </is>
-      </c>
+          <t>Longevity Commitment (yr) typ</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr"/>
       <c r="D173" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E173" s="4" t="inlineStr">
-        <is>
-          <t>CHANGED</t>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E173" s="3" t="inlineStr">
+        <is>
+          <t>ADDED_COLUMN</t>
         </is>
       </c>
     </row>
@@ -4242,67 +4220,59 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Timers (16-bit) typ</t>
-        </is>
-      </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>3, 5</t>
-        </is>
-      </c>
+          <t>Longevity Starting Date</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr"/>
       <c r="D174" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E174" s="5" t="inlineStr">
-        <is>
-          <t>DATASHEET_OVERRIDES_API</t>
+          <t>2026-01-01T00:00:00.000+01:00</t>
+        </is>
+      </c>
+      <c r="E174" s="3" t="inlineStr">
+        <is>
+          <t>ADDED_COLUMN</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>STM32WB55VE</t>
+          <t>STM32WB55CC</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Timers (16-bit) typ</t>
-        </is>
-      </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>3||5 (workbook and API agree)</t>
-        </is>
-      </c>
+          <t>Longevity Commitment (yr) typ</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr"/>
       <c r="D175" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E175" s="6" t="inlineStr">
-        <is>
-          <t>ORIGINAL_MATCHED_API_NOT_DATASHEET</t>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E175" s="3" t="inlineStr">
+        <is>
+          <t>ADDED_COLUMN</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>STM32WB55VE</t>
+          <t>STM32WB55CC</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Longevity Commitment (yr) typ</t>
+          <t>Longevity Starting Date</t>
         </is>
       </c>
       <c r="C176" t="inlineStr"/>
       <c r="D176" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2026-01-01T00:00:00.000+01:00</t>
         </is>
       </c>
       <c r="E176" s="3" t="inlineStr">
@@ -4314,18 +4284,18 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>STM32WB55VE</t>
+          <t>STM32WB55RE</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Longevity Starting Date</t>
+          <t>Longevity Commitment (yr) typ</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
       <c r="D177" t="inlineStr">
         <is>
-          <t>2026-01-01T00:00:00.000+01:00</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E177" s="3" t="inlineStr">
@@ -4337,18 +4307,18 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>STM32WB55CC</t>
+          <t>STM32WB55RE</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Longevity Commitment (yr) typ</t>
+          <t>Longevity Starting Date</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
       <c r="D178" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2026-01-01T00:00:00.000+01:00</t>
         </is>
       </c>
       <c r="E178" s="3" t="inlineStr">
@@ -4360,18 +4330,18 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>STM32WB55CC</t>
+          <t>STM32WB55VC</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Longevity Starting Date</t>
+          <t>Longevity Commitment (yr) typ</t>
         </is>
       </c>
       <c r="C179" t="inlineStr"/>
       <c r="D179" t="inlineStr">
         <is>
-          <t>2026-01-01T00:00:00.000+01:00</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E179" s="3" t="inlineStr">
@@ -4383,18 +4353,18 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>STM32WB55RE</t>
+          <t>STM32WB55VC</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Longevity Commitment (yr) typ</t>
+          <t>Longevity Starting Date</t>
         </is>
       </c>
       <c r="C180" t="inlineStr"/>
       <c r="D180" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2026-01-01T00:00:00.000+01:00</t>
         </is>
       </c>
       <c r="E180" s="3" t="inlineStr">
@@ -4406,18 +4376,18 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>STM32WB55RE</t>
+          <t>STM32WB55CG</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Longevity Starting Date</t>
+          <t>Longevity Commitment (yr) typ</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
       <c r="D181" t="inlineStr">
         <is>
-          <t>2026-01-01T00:00:00.000+01:00</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E181" s="3" t="inlineStr">
@@ -4429,88 +4399,76 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>STM32WB55VC</t>
+          <t>STM32WB55CG</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Timers (16-bit) typ</t>
-        </is>
-      </c>
-      <c r="C182" t="inlineStr">
-        <is>
-          <t>3||5</t>
-        </is>
-      </c>
+          <t>Longevity Starting Date</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr"/>
       <c r="D182" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E182" s="4" t="inlineStr">
-        <is>
-          <t>CHANGED</t>
+          <t>2026-01-01T00:00:00.000+01:00</t>
+        </is>
+      </c>
+      <c r="E182" s="3" t="inlineStr">
+        <is>
+          <t>ADDED_COLUMN</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>STM32WB55VC</t>
+          <t>STM32WB55RG</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Timers (16-bit) typ</t>
-        </is>
-      </c>
-      <c r="C183" t="inlineStr">
-        <is>
-          <t>3, 5</t>
-        </is>
-      </c>
+          <t>Longevity Commitment (yr) typ</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr"/>
       <c r="D183" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E183" s="5" t="inlineStr">
-        <is>
-          <t>DATASHEET_OVERRIDES_API</t>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E183" s="3" t="inlineStr">
+        <is>
+          <t>ADDED_COLUMN</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>STM32WB55VC</t>
+          <t>STM32WB55RG</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Timers (16-bit) typ</t>
-        </is>
-      </c>
-      <c r="C184" t="inlineStr">
-        <is>
-          <t>3||5 (workbook and API agree)</t>
-        </is>
-      </c>
+          <t>Longevity Starting Date</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr"/>
       <c r="D184" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E184" s="6" t="inlineStr">
-        <is>
-          <t>ORIGINAL_MATCHED_API_NOT_DATASHEET</t>
+          <t>2026-01-01T00:00:00.000+01:00</t>
+        </is>
+      </c>
+      <c r="E184" s="3" t="inlineStr">
+        <is>
+          <t>ADDED_COLUMN</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>STM32WB55VC</t>
+          <t>STM32WB35CE</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4533,7 +4491,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>STM32WB55VC</t>
+          <t>STM32WB35CE</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4556,7 +4514,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>STM32WB55CG</t>
+          <t>STM32WB35CC</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -4579,7 +4537,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>STM32WB55CG</t>
+          <t>STM32WB35CC</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -4602,7 +4560,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>STM32WB55RG</t>
+          <t>STM32WB55CE</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -4625,7 +4583,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>STM32WB55RG</t>
+          <t>STM32WB55CE</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -4648,7 +4606,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>STM32WB35CE</t>
+          <t>STM32WB06CC</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -4671,7 +4629,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>STM32WB35CE</t>
+          <t>STM32WB06CC</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -4694,7 +4652,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>STM32WB35CC</t>
+          <t>STM32WB09KE</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -4717,7 +4675,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>STM32WB35CC</t>
+          <t>STM32WB09KE</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -4740,7 +4698,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>STM32WB55CE</t>
+          <t>STM32WB05KZ</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -4763,7 +4721,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>STM32WB55CE</t>
+          <t>STM32WB05KZ</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -4786,7 +4744,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>STM32WB06CC</t>
+          <t>STM32WB06KC</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -4809,7 +4767,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>STM32WB06CC</t>
+          <t>STM32WB06KC</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -4832,7 +4790,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>STM32WB09KE</t>
+          <t>STM32WB07CC</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -4855,7 +4813,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>STM32WB09KE</t>
+          <t>STM32WB07CC</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -4878,7 +4836,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>STM32WB05KZ</t>
+          <t>STM32WB05TZ</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -4901,7 +4859,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>STM32WB05KZ</t>
+          <t>STM32WB05TZ</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -4924,7 +4882,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>STM32WB06KC</t>
+          <t>STM32WB07KC</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -4947,7 +4905,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>STM32WB06KC</t>
+          <t>STM32WB07KC</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -4970,41 +4928,45 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>STM32WB07CC</t>
+          <t>STM32WB05KN</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Longevity Commitment (yr) typ</t>
-        </is>
-      </c>
-      <c r="C205" t="inlineStr"/>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E205" s="3" t="inlineStr">
-        <is>
-          <t>ADDED_COLUMN</t>
+          <t>Arm Cortex-M0+</t>
+        </is>
+      </c>
+      <c r="E205" s="4" t="inlineStr">
+        <is>
+          <t>BLANK_FILLED</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>STM32WB07CC</t>
+          <t>STM32WB05KN</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Longevity Starting Date</t>
+          <t>Longevity Commitment (yr) typ</t>
         </is>
       </c>
       <c r="C206" t="inlineStr"/>
       <c r="D206" t="inlineStr">
         <is>
-          <t>2026-01-01T00:00:00.000+01:00</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E206" s="3" t="inlineStr">
@@ -5016,18 +4978,18 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>STM32WB05TZ</t>
+          <t>STM32WB05KN</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Longevity Commitment (yr) typ</t>
+          <t>Longevity Starting Date</t>
         </is>
       </c>
       <c r="C207" t="inlineStr"/>
       <c r="D207" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2026-01-01T00:00:00.000+01:00</t>
         </is>
       </c>
       <c r="E207" s="3" t="inlineStr">
@@ -5039,18 +5001,18 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>STM32WB05TZ</t>
+          <t>STM32WB09TE</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Longevity Starting Date</t>
+          <t>Longevity Commitment (yr) typ</t>
         </is>
       </c>
       <c r="C208" t="inlineStr"/>
       <c r="D208" t="inlineStr">
         <is>
-          <t>2026-01-01T00:00:00.000+01:00</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E208" s="3" t="inlineStr">
@@ -5062,18 +5024,18 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>STM32WB07KC</t>
+          <t>STM32WB09TE</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Longevity Commitment (yr) typ</t>
+          <t>Longevity Starting Date</t>
         </is>
       </c>
       <c r="C209" t="inlineStr"/>
       <c r="D209" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2026-01-01T00:00:00.000+01:00</t>
         </is>
       </c>
       <c r="E209" s="3" t="inlineStr">
@@ -5085,18 +5047,18 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>STM32WB07KC</t>
+          <t>STM32WB05TN</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Longevity Starting Date</t>
+          <t>Longevity Commitment (yr) typ</t>
         </is>
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="inlineStr">
         <is>
-          <t>2026-01-01T00:00:00.000+01:00</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E210" s="3" t="inlineStr">
@@ -5108,197 +5070,28 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>STM32WB05KN</t>
+          <t>STM32WB05TN</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="C211" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>Longevity Starting Date</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr"/>
       <c r="D211" t="inlineStr">
         <is>
-          <t>Arm Cortex-M0+</t>
-        </is>
-      </c>
-      <c r="E211" s="7" t="inlineStr">
-        <is>
-          <t>BLANK_FILLED</t>
-        </is>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" t="inlineStr">
-        <is>
-          <t>STM32WB05KN</t>
-        </is>
-      </c>
-      <c r="B212" t="inlineStr">
-        <is>
-          <t>Longevity Commitment (yr) typ</t>
-        </is>
-      </c>
-      <c r="C212" t="inlineStr"/>
-      <c r="D212" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E212" s="3" t="inlineStr">
-        <is>
-          <t>ADDED_COLUMN</t>
-        </is>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" t="inlineStr">
-        <is>
-          <t>STM32WB05KN</t>
-        </is>
-      </c>
-      <c r="B213" t="inlineStr">
-        <is>
-          <t>Longevity Starting Date</t>
-        </is>
-      </c>
-      <c r="C213" t="inlineStr"/>
-      <c r="D213" t="inlineStr">
-        <is>
-          <t>2026-01-01T00:00:00.000+01:00</t>
-        </is>
-      </c>
-      <c r="E213" s="3" t="inlineStr">
-        <is>
-          <t>ADDED_COLUMN</t>
-        </is>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" t="inlineStr">
-        <is>
-          <t>STM32WB09TE</t>
-        </is>
-      </c>
-      <c r="B214" t="inlineStr">
-        <is>
-          <t>Longevity Commitment (yr) typ</t>
-        </is>
-      </c>
-      <c r="C214" t="inlineStr"/>
-      <c r="D214" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E214" s="3" t="inlineStr">
-        <is>
-          <t>ADDED_COLUMN</t>
-        </is>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" t="inlineStr">
-        <is>
-          <t>STM32WB09TE</t>
-        </is>
-      </c>
-      <c r="B215" t="inlineStr">
-        <is>
-          <t>Longevity Starting Date</t>
-        </is>
-      </c>
-      <c r="C215" t="inlineStr"/>
-      <c r="D215" t="inlineStr">
-        <is>
-          <t>2026-01-01T00:00:00.000+01:00</t>
-        </is>
-      </c>
-      <c r="E215" s="3" t="inlineStr">
-        <is>
-          <t>ADDED_COLUMN</t>
-        </is>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" t="inlineStr">
-        <is>
-          <t>STM32WB05TN</t>
-        </is>
-      </c>
-      <c r="B216" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="C216" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D216" t="inlineStr">
-        <is>
-          <t>Arm Cortex-M0+</t>
-        </is>
-      </c>
-      <c r="E216" s="7" t="inlineStr">
-        <is>
-          <t>BLANK_FILLED</t>
-        </is>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" t="inlineStr">
-        <is>
-          <t>STM32WB05TN</t>
-        </is>
-      </c>
-      <c r="B217" t="inlineStr">
-        <is>
-          <t>Longevity Commitment (yr) typ</t>
-        </is>
-      </c>
-      <c r="C217" t="inlineStr"/>
-      <c r="D217" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E217" s="3" t="inlineStr">
-        <is>
-          <t>ADDED_COLUMN</t>
-        </is>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" t="inlineStr">
-        <is>
-          <t>STM32WB05TN</t>
-        </is>
-      </c>
-      <c r="B218" t="inlineStr">
-        <is>
-          <t>Longevity Starting Date</t>
-        </is>
-      </c>
-      <c r="C218" t="inlineStr"/>
-      <c r="D218" t="inlineStr">
-        <is>
-          <t>2026-01-01T00:00:00.000+01:00</t>
-        </is>
-      </c>
-      <c r="E218" s="3" t="inlineStr">
+          <t>2026-01-01T00:00:00.000+01:00</t>
+        </is>
+      </c>
+      <c r="E211" s="3" t="inlineStr">
         <is>
           <t>ADDED_COLUMN</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A18:E218"/>
+  <autoFilter ref="A18:E211"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>